<commit_message>
update ARPD and plots
</commit_message>
<xml_diff>
--- a/output/statistical_tests.xlsx
+++ b/output/statistical_tests.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Statistical Tests" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Statistical Tests" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16,9 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="+0.0000;-0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.00&quot;%&quot;"/>
+    <numFmt numFmtId="167" formatCode="+0.00&quot;%&quot;;-0.00&quot;%&quot;"/>
   </numFmts>
   <fonts count="3">
     <font>
@@ -39,7 +41,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="12">
+  <fills count="14">
     <fill>
       <patternFill/>
     </fill>
@@ -79,6 +81,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEEFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDFFDD"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,7 +135,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -149,19 +161,37 @@
     <xf numFmtId="165" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="2" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="2" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -529,7 +559,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:S12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -541,13 +571,16 @@
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="13" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
     <col width="11" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -596,37 +629,52 @@
           <t>Δ mean (MA−MH)</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>ARPD MH (%)</t>
+        </is>
+      </c>
+      <c r="K1" s="3" t="inlineStr">
+        <is>
+          <t>ARPD Memetic (%)</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>ΔARPD (MA−MH)</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Wilcoxon stat</t>
         </is>
       </c>
-      <c r="K1" s="4" t="inlineStr">
+      <c r="N1" s="4" t="inlineStr">
         <is>
           <t>Wilcoxon p</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>Sig. (W)</t>
         </is>
       </c>
-      <c r="M1" s="5" t="inlineStr">
+      <c r="P1" s="5" t="inlineStr">
         <is>
           <t>Paired t stat</t>
         </is>
       </c>
-      <c r="N1" s="5" t="inlineStr">
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>Paired t p</t>
         </is>
       </c>
-      <c r="O1" s="5" t="inlineStr">
+      <c r="R1" s="5" t="inlineStr">
         <is>
           <t>Sig. (t)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Conclusion</t>
         </is>
@@ -664,89 +712,107 @@
       <c r="I2" s="8" t="n">
         <v>-0.09999999999999964</v>
       </c>
-      <c r="J2" s="7" t="n">
+      <c r="J2" s="9" t="n">
+        <v>11.11111111111111</v>
+      </c>
+      <c r="K2" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="L2" s="11" t="n">
+        <v>-1.111111111111111</v>
+      </c>
+      <c r="M2" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="K2" s="7" t="n">
+      <c r="N2" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="L2" s="9" t="inlineStr">
+      <c r="O2" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="M2" s="7" t="n">
+      <c r="P2" s="7" t="n">
         <v>0.5570860145311556</v>
       </c>
-      <c r="N2" s="7" t="n">
-        <v>0.5910512317836045</v>
-      </c>
-      <c r="O2" s="9" t="inlineStr">
+      <c r="Q2" s="7" t="n">
+        <v>0.5910512317836047</v>
+      </c>
+      <c r="R2" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="P2" s="9" t="inlineStr">
+      <c r="S2" s="12" t="inlineStr">
         <is>
           <t>no sig. diff.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="10" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>2M46 (46 ops)</t>
         </is>
       </c>
-      <c r="B3" s="10" t="inlineStr">
+      <c r="B3" s="13" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="C3" s="11" t="n">
+      <c r="C3" s="14" t="n">
         <v>16.6</v>
       </c>
-      <c r="D3" s="11" t="n">
+      <c r="D3" s="14" t="n">
         <v>0.4898979485566356</v>
       </c>
-      <c r="E3" s="11" t="n">
+      <c r="E3" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="F3" s="11" t="n">
+      <c r="F3" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="G3" s="11" t="n">
+      <c r="G3" s="14" t="n">
         <v>0.6324555320336759</v>
       </c>
-      <c r="H3" s="11" t="n">
+      <c r="H3" s="14" t="n">
         <v>15</v>
       </c>
       <c r="I3" s="8" t="n">
         <v>-0.6000000000000014</v>
       </c>
-      <c r="J3" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" s="11" t="n">
+      <c r="J3" s="9" t="n">
+        <v>10.66666666666667</v>
+      </c>
+      <c r="K3" s="10" t="n">
+        <v>6.666666666666667</v>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>-4.000000000000001</v>
+      </c>
+      <c r="M3" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" s="14" t="n">
         <v>0.0625</v>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="O3" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="M3" s="11" t="n">
+      <c r="P3" s="14" t="n">
         <v>2.713602101199872</v>
       </c>
-      <c r="N3" s="11" t="n">
-        <v>0.02385638454012205</v>
-      </c>
-      <c r="O3" s="12" t="inlineStr">
+      <c r="Q3" s="14" t="n">
+        <v>0.02385638454012203</v>
+      </c>
+      <c r="R3" s="15" t="inlineStr">
         <is>
           <t>*   p&lt;0.05</t>
         </is>
       </c>
-      <c r="P3" s="12" t="inlineStr">
+      <c r="S3" s="15" t="inlineStr">
         <is>
           <t>Memetic better (1/2 tests)</t>
         </is>
@@ -784,89 +850,107 @@
       <c r="I4" s="8" t="n">
         <v>-0.8000000000000043</v>
       </c>
-      <c r="J4" s="7" t="n">
+      <c r="J4" s="9" t="n">
+        <v>8.205128205128204</v>
+      </c>
+      <c r="K4" s="10" t="n">
+        <v>6.153846153846154</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>-2.05128205128205</v>
+      </c>
+      <c r="M4" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="K4" s="7" t="n">
+      <c r="N4" s="7" t="n">
         <v>0.4296875</v>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="O4" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="M4" s="7" t="n">
+      <c r="P4" s="7" t="n">
         <v>1.017826715615965</v>
       </c>
-      <c r="N4" s="7" t="n">
-        <v>0.3353398249453193</v>
-      </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="Q4" s="7" t="n">
+        <v>0.335339824945319</v>
+      </c>
+      <c r="R4" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="P4" s="9" t="inlineStr">
+      <c r="S4" s="12" t="inlineStr">
         <is>
           <t>no sig. diff.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="10" t="inlineStr">
+      <c r="A5" s="13" t="inlineStr">
         <is>
           <t>6M163 (163 ops)</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C5" s="14" t="n">
         <v>55.4</v>
       </c>
-      <c r="D5" s="11" t="n">
+      <c r="D5" s="14" t="n">
         <v>1.496662954709577</v>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="14" t="n">
         <v>52</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="14" t="n">
         <v>53.7</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="14" t="n">
         <v>0.6403124237432849</v>
       </c>
-      <c r="H5" s="11" t="n">
+      <c r="H5" s="14" t="n">
         <v>53</v>
       </c>
       <c r="I5" s="8" t="n">
         <v>-1.699999999999996</v>
       </c>
-      <c r="J5" s="11" t="n">
+      <c r="J5" s="9" t="n">
+        <v>6.538461538461538</v>
+      </c>
+      <c r="K5" s="10" t="n">
+        <v>3.269230769230769</v>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>-3.26923076923077</v>
+      </c>
+      <c r="M5" s="14" t="n">
         <v>4.5</v>
       </c>
-      <c r="K5" s="11" t="n">
+      <c r="N5" s="14" t="n">
         <v>0.03125</v>
       </c>
-      <c r="L5" s="12" t="inlineStr">
+      <c r="O5" s="15" t="inlineStr">
         <is>
           <t>*   p&lt;0.05</t>
         </is>
       </c>
-      <c r="M5" s="11" t="n">
+      <c r="P5" s="14" t="n">
         <v>2.939591130291598</v>
       </c>
-      <c r="N5" s="11" t="n">
+      <c r="Q5" s="14" t="n">
         <v>0.01649769830177924</v>
       </c>
-      <c r="O5" s="12" t="inlineStr">
+      <c r="R5" s="15" t="inlineStr">
         <is>
           <t>*   p&lt;0.05</t>
         </is>
       </c>
-      <c r="P5" s="12" t="inlineStr">
+      <c r="S5" s="15" t="inlineStr">
         <is>
           <t>Memetic better</t>
         </is>
@@ -901,92 +985,110 @@
       <c r="H6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v/>
-      </c>
-      <c r="K6" s="7" t="n">
-        <v/>
-      </c>
-      <c r="L6" s="9" t="inlineStr">
+      <c r="I6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v/>
+      </c>
+      <c r="K6" s="10" t="n">
+        <v/>
+      </c>
+      <c r="L6" s="17" t="n">
+        <v/>
+      </c>
+      <c r="M6" s="7" t="n">
+        <v/>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v/>
+      </c>
+      <c r="O6" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="M6" s="7" t="n">
-        <v/>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v/>
-      </c>
-      <c r="O6" s="9" t="inlineStr">
+      <c r="P6" s="7" t="n">
+        <v/>
+      </c>
+      <c r="Q6" s="7" t="n">
+        <v/>
+      </c>
+      <c r="R6" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="P6" s="9" t="inlineStr">
+      <c r="S6" s="12" t="inlineStr">
         <is>
           <t>identical</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="10" t="inlineStr">
+      <c r="A7" s="13" t="inlineStr">
         <is>
           <t>6M140 n=25</t>
         </is>
       </c>
-      <c r="B7" s="10" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Table 8</t>
         </is>
       </c>
-      <c r="C7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <v/>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v/>
-      </c>
-      <c r="L7" s="9" t="inlineStr">
+      <c r="C7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v/>
+      </c>
+      <c r="K7" s="10" t="n">
+        <v/>
+      </c>
+      <c r="L7" s="18" t="n">
+        <v/>
+      </c>
+      <c r="M7" s="14" t="n">
+        <v/>
+      </c>
+      <c r="N7" s="14" t="n">
+        <v/>
+      </c>
+      <c r="O7" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="M7" s="11" t="n">
-        <v/>
-      </c>
-      <c r="N7" s="11" t="n">
-        <v/>
-      </c>
-      <c r="O7" s="9" t="inlineStr">
+      <c r="P7" s="14" t="n">
+        <v/>
+      </c>
+      <c r="Q7" s="14" t="n">
+        <v/>
+      </c>
+      <c r="R7" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="P7" s="9" t="inlineStr">
+      <c r="S7" s="12" t="inlineStr">
         <is>
           <t>identical</t>
         </is>
@@ -1021,92 +1123,110 @@
       <c r="H8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="I8" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v/>
-      </c>
-      <c r="K8" s="7" t="n">
-        <v/>
-      </c>
-      <c r="L8" s="9" t="inlineStr">
+      <c r="I8" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v/>
+      </c>
+      <c r="K8" s="10" t="n">
+        <v/>
+      </c>
+      <c r="L8" s="17" t="n">
+        <v/>
+      </c>
+      <c r="M8" s="7" t="n">
+        <v/>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v/>
+      </c>
+      <c r="O8" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="M8" s="7" t="n">
-        <v/>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v/>
-      </c>
-      <c r="O8" s="9" t="inlineStr">
+      <c r="P8" s="7" t="n">
+        <v/>
+      </c>
+      <c r="Q8" s="7" t="n">
+        <v/>
+      </c>
+      <c r="R8" s="12" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="P8" s="9" t="inlineStr">
+      <c r="S8" s="12" t="inlineStr">
         <is>
           <t>identical</t>
         </is>
       </c>
     </row>
     <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="10" t="inlineStr">
+      <c r="A9" s="13" t="inlineStr">
         <is>
           <t>6M140 n=60</t>
         </is>
       </c>
-      <c r="B9" s="10" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>Table 8</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n">
+      <c r="C9" s="14" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="D9" s="11" t="n">
+      <c r="D9" s="14" t="n">
         <v>0.4</v>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="14" t="n">
         <v>9.6</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="G9" s="14" t="n">
         <v>0.4898979485566356</v>
       </c>
-      <c r="H9" s="11" t="n">
+      <c r="H9" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="I9" s="13" t="n">
+      <c r="I9" s="16" t="n">
         <v>0.4000000000000004</v>
       </c>
-      <c r="J9" s="11" t="n">
+      <c r="J9" s="9" t="n">
+        <v>2.222222222222222</v>
+      </c>
+      <c r="K9" s="10" t="n">
+        <v>6.666666666666666</v>
+      </c>
+      <c r="L9" s="19" t="n">
+        <v>4.444444444444444</v>
+      </c>
+      <c r="M9" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="K9" s="11" t="n">
+      <c r="N9" s="14" t="n">
         <v>0.2890625</v>
       </c>
-      <c r="L9" s="9" t="inlineStr">
+      <c r="O9" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="M9" s="11" t="n">
+      <c r="P9" s="14" t="n">
         <v>-1.5</v>
       </c>
-      <c r="N9" s="11" t="n">
-        <v>0.1678506560570751</v>
-      </c>
-      <c r="O9" s="9" t="inlineStr">
+      <c r="Q9" s="14" t="n">
+        <v>0.1678506560570749</v>
+      </c>
+      <c r="R9" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="P9" s="9" t="inlineStr">
+      <c r="S9" s="12" t="inlineStr">
         <is>
           <t>no sig. diff.</t>
         </is>
@@ -1141,92 +1261,110 @@
       <c r="H10" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="I10" s="13" t="n">
+      <c r="I10" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="9" t="n">
+        <v>6.842105263157895</v>
+      </c>
+      <c r="K10" s="10" t="n">
+        <v>9.473684210526315</v>
+      </c>
+      <c r="L10" s="19" t="n">
+        <v>2.63157894736842</v>
+      </c>
+      <c r="M10" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="K10" s="7" t="n">
+      <c r="N10" s="7" t="n">
         <v>0.12109375</v>
       </c>
-      <c r="L10" s="9" t="inlineStr">
+      <c r="O10" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="M10" s="7" t="n">
+      <c r="P10" s="7" t="n">
         <v>-0.9583148474999098</v>
       </c>
-      <c r="N10" s="7" t="n">
-        <v>0.3629382386791292</v>
-      </c>
-      <c r="O10" s="9" t="inlineStr">
+      <c r="Q10" s="7" t="n">
+        <v>0.3629382386791291</v>
+      </c>
+      <c r="R10" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="P10" s="9" t="inlineStr">
+      <c r="S10" s="12" t="inlineStr">
         <is>
           <t>no sig. diff.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="10" t="inlineStr">
+      <c r="A11" s="13" t="inlineStr">
         <is>
           <t>6M140 n=120</t>
         </is>
       </c>
-      <c r="B11" s="10" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Table 8</t>
         </is>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C11" s="14" t="n">
         <v>36.4</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D11" s="14" t="n">
         <v>1.907878402833892</v>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="14" t="n">
         <v>33.9</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="14" t="n">
         <v>0.5385164807134504</v>
       </c>
-      <c r="H11" s="11" t="n">
+      <c r="H11" s="14" t="n">
         <v>33</v>
       </c>
       <c r="I11" s="8" t="n">
         <v>-2.5</v>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="J11" s="9" t="n">
+        <v>10.3030303030303</v>
+      </c>
+      <c r="K11" s="10" t="n">
+        <v>2.727272727272728</v>
+      </c>
+      <c r="L11" s="11" t="n">
+        <v>-7.575757575757575</v>
+      </c>
+      <c r="M11" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="K11" s="11" t="n">
+      <c r="N11" s="14" t="n">
         <v>0.015625</v>
       </c>
-      <c r="L11" s="12" t="inlineStr">
+      <c r="O11" s="15" t="inlineStr">
         <is>
           <t>*   p&lt;0.05</t>
         </is>
       </c>
-      <c r="M11" s="11" t="n">
+      <c r="P11" s="14" t="n">
         <v>3.337456196174886</v>
       </c>
-      <c r="N11" s="11" t="n">
-        <v>0.008695290574962428</v>
-      </c>
-      <c r="O11" s="12" t="inlineStr">
+      <c r="Q11" s="14" t="n">
+        <v>0.008695290574962418</v>
+      </c>
+      <c r="R11" s="15" t="inlineStr">
         <is>
           <t>**  p&lt;0.01</t>
         </is>
       </c>
-      <c r="P11" s="12" t="inlineStr">
+      <c r="S11" s="15" t="inlineStr">
         <is>
           <t>Memetic better</t>
         </is>
@@ -1264,29 +1402,38 @@
       <c r="I12" s="8" t="n">
         <v>-0.8000000000000043</v>
       </c>
-      <c r="J12" s="7" t="n">
+      <c r="J12" s="9" t="n">
+        <v>8.205128205128204</v>
+      </c>
+      <c r="K12" s="10" t="n">
+        <v>6.153846153846154</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <v>-2.05128205128205</v>
+      </c>
+      <c r="M12" s="7" t="n">
         <v>12</v>
       </c>
-      <c r="K12" s="7" t="n">
+      <c r="N12" s="7" t="n">
         <v>0.4296875</v>
       </c>
-      <c r="L12" s="9" t="inlineStr">
+      <c r="O12" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="M12" s="7" t="n">
+      <c r="P12" s="7" t="n">
         <v>1.017826715615965</v>
       </c>
-      <c r="N12" s="7" t="n">
-        <v>0.3353398249453193</v>
-      </c>
-      <c r="O12" s="9" t="inlineStr">
+      <c r="Q12" s="7" t="n">
+        <v>0.335339824945319</v>
+      </c>
+      <c r="R12" s="12" t="inlineStr">
         <is>
           <t>n.s.</t>
         </is>
       </c>
-      <c r="P12" s="9" t="inlineStr">
+      <c r="S12" s="12" t="inlineStr">
         <is>
           <t>no sig. diff.</t>
         </is>

</xml_diff>